<commit_message>
Add forecasting pipeline with lost sales correction
- run_forecasting.py: full pipeline for all 12 product categories
  (LSC → MAPE ensemble → channel × size forecast → Excel export)
- lost_sales_correction.py: hierarchical correction (3 levels),
  data-driven channel clusters via Pearson correlation
- tune_ma_window.py / tune_ses_alpha.py: global parameter tuning
  across all categories (MA=3, α=0.47)
- data/PPP_stu_product_categories.xlsx: official category definitions
- Remove old per-category forecasting scripts

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/PPP_stu_products.xlsx
+++ b/data/PPP_stu_products.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maximilianlangenau/Library/Mobile Documents/com~apple~CloudDocs/Master/Gent/UGent/Semester 4/Supply Chain Management/Group Assignment/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maximilianlangenau/PycharmProjects/Supply Chain Management/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD68BC59-B192-F049-A1F1-E8B78A957299}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="17100" windowHeight="19820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="17100" windowHeight="19780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -341,6 +341,7 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">

</xml_diff>